<commit_message>
Improve workbook coordinate fallback
Co-authored-by: hhousni <63563021+hhousni@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/masters/master_town_village.xlsx
+++ b/masters/master_town_village.xlsx
@@ -795,8 +795,12 @@
           <t>BARAKANI</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>-12.13923932658967</v>
+      </c>
+      <c r="H11" t="n">
+        <v>44.43117532297685</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1266,10 +1270,10 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>-12.3491749</v>
+        <v>-12.3201731</v>
       </c>
       <c r="H24" t="n">
-        <v>43.8222246</v>
+        <v>44.4731801</v>
       </c>
     </row>
     <row r="25">
@@ -2079,8 +2083,12 @@
           <t>BARAKANI</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="G47" t="n">
+        <v>-12.13923932658967</v>
+      </c>
+      <c r="H47" t="n">
+        <v>44.43117532297685</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3358,10 +3366,10 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>-12.3491749</v>
+        <v>-12.3201731</v>
       </c>
       <c r="H82" t="n">
-        <v>43.8222246</v>
+        <v>44.4731801</v>
       </c>
     </row>
     <row r="83">
@@ -4233,8 +4241,12 @@
           <t>MILEMBENI</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="G106" t="n">
+        <v>-12.20224155888374</v>
+      </c>
+      <c r="H106" t="n">
+        <v>44.26310520358714</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7921,7 +7933,7 @@
         <v>-11.88428639896506</v>
       </c>
       <c r="H206" t="n">
-        <v>43.49101856641398</v>
+        <v>43.49101856641399</v>
       </c>
     </row>
     <row r="207">
@@ -12767,8 +12779,12 @@
           <t>MILEMBENI</t>
         </is>
       </c>
-      <c r="G337" t="inlineStr"/>
-      <c r="H337" t="inlineStr"/>
+      <c r="G337" t="n">
+        <v>-12.20224155888374</v>
+      </c>
+      <c r="H337" t="n">
+        <v>44.26310520358714</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">

</xml_diff>